<commit_message>
Update inventory quantities and items
</commit_message>
<xml_diff>
--- a/Inventory.xlsx
+++ b/Inventory.xlsx
@@ -78,17 +78,17 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="InventoryTable" displayName="InventoryTable" ref="A1:F6" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="6">
-    <x:tableColumn id="1" name="Item ID"/>
-    <x:tableColumn id="2" name="Item Name"/>
-    <x:tableColumn id="3" name="Category"/>
-    <x:tableColumn id="4" name="Quantity"/>
-    <x:tableColumn id="5" name="Location"/>
-    <x:tableColumn id="6" name="Status"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</x:table>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="InventoryTable" displayName="InventoryTable" ref="A1:F8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <tableColumns count="6">
+    <tableColumn id="1" name="Item ID"/>
+    <tableColumn id="2" name="Item Name"/>
+    <tableColumn id="3" name="Category"/>
+    <tableColumn id="4" name="Quantity"/>
+    <tableColumn id="5" name="Location"/>
+    <tableColumn id="6" name="Status"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -283,141 +283,181 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="10" t="str">
-        <x:v>Item ID</x:v>
-      </x:c>
-      <x:c r="B1" s="10" t="str">
-        <x:v>Item Name</x:v>
-      </x:c>
-      <x:c r="C1" s="10" t="str">
-        <x:v>Category</x:v>
-      </x:c>
-      <x:c r="D1" s="10" t="str">
-        <x:v>Quantity</x:v>
-      </x:c>
-      <x:c r="E1" s="10" t="str">
-        <x:v>Location</x:v>
-      </x:c>
-      <x:c r="F1" s="10" t="str">
-        <x:v>Status</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2">
-      <x:c r="A2" s="11" t="str">
-        <x:v>INV001</x:v>
-      </x:c>
-      <x:c r="B2" s="11" t="str">
-        <x:v>Laptop</x:v>
-      </x:c>
-      <x:c r="C2" s="11" t="str">
-        <x:v>IT Equipment</x:v>
-      </x:c>
-      <x:c r="D2" s="11" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="E2" s="11" t="str">
-        <x:v>Bangalore</x:v>
-      </x:c>
-      <x:c r="F2" s="11" t="str">
-        <x:v>Available</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="11" t="str">
-        <x:v>INV002</x:v>
-      </x:c>
-      <x:c r="B3" s="11" t="str">
-        <x:v>Monitor</x:v>
-      </x:c>
-      <x:c r="C3" s="11" t="str">
-        <x:v>IT Equipment</x:v>
-      </x:c>
-      <x:c r="D3" s="11" t="n">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="E3" s="11" t="str">
-        <x:v>Bangalore</x:v>
-      </x:c>
-      <x:c r="F3" s="11" t="str">
-        <x:v>Available</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="11" t="str">
-        <x:v>INV003</x:v>
-      </x:c>
-      <x:c r="B4" s="11" t="str">
-        <x:v>Keyboard</x:v>
-      </x:c>
-      <x:c r="C4" s="11" t="str">
-        <x:v>Accessories</x:v>
-      </x:c>
-      <x:c r="D4" s="11" t="n">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="E4" s="11" t="str">
-        <x:v>Hyderabad</x:v>
-      </x:c>
-      <x:c r="F4" s="11" t="str">
-        <x:v>Available</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="11" t="str">
-        <x:v>INV004</x:v>
-      </x:c>
-      <x:c r="B5" s="11" t="str">
-        <x:v>Mouse</x:v>
-      </x:c>
-      <x:c r="C5" s="11" t="str">
-        <x:v>Accessories</x:v>
-      </x:c>
-      <x:c r="D5" s="11" t="n">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="E5" s="11" t="str">
-        <x:v>Pune</x:v>
-      </x:c>
-      <x:c r="F5" s="11" t="str">
-        <x:v>Available</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="11" t="str">
-        <x:v>INV005</x:v>
-      </x:c>
-      <x:c r="B6" s="11" t="str">
-        <x:v>Printer</x:v>
-      </x:c>
-      <x:c r="C6" s="11" t="str">
-        <x:v>Office Equipment</x:v>
-      </x:c>
-      <x:c r="D6" s="11" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="E6" s="11" t="str">
-        <x:v>Chennai</x:v>
-      </x:c>
-      <x:c r="F6" s="11" t="str">
-        <x:v>Available</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R65794bffdeb745ea"/>
-  </x:tableParts>
-</x:worksheet>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="20" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="12" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="16" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="14" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="str">
+        <v>Item ID</v>
+      </c>
+      <c r="B1" s="10" t="str">
+        <v>Item Name</v>
+      </c>
+      <c r="C1" s="10" t="str">
+        <v>Category</v>
+      </c>
+      <c r="D1" s="10" t="str">
+        <v>Quantity</v>
+      </c>
+      <c r="E1" s="10" t="str">
+        <v>Location</v>
+      </c>
+      <c r="F1" s="10" t="str">
+        <v>Status</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="11" t="str">
+        <v>INV001</v>
+      </c>
+      <c r="B2" s="11" t="str">
+        <v>Laptop</v>
+      </c>
+      <c r="C2" s="11" t="str">
+        <v>IT Equipment</v>
+      </c>
+      <c r="D2" s="11" t="n">
+        <v>15</v>
+      </c>
+      <c r="E2" s="11" t="str">
+        <v>Bangalore</v>
+      </c>
+      <c r="F2" s="11" t="str">
+        <v>Available</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="11" t="str">
+        <v>INV002</v>
+      </c>
+      <c r="B3" s="11" t="str">
+        <v>Monitor</v>
+      </c>
+      <c r="C3" s="11" t="str">
+        <v>IT Equipment</v>
+      </c>
+      <c r="D3" s="11" t="n">
+        <v>25</v>
+      </c>
+      <c r="E3" s="11" t="str">
+        <v>Bangalore</v>
+      </c>
+      <c r="F3" s="11" t="str">
+        <v>Available</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="str">
+        <v>INV003</v>
+      </c>
+      <c r="B4" s="11" t="str">
+        <v>Keyboard</v>
+      </c>
+      <c r="C4" s="11" t="str">
+        <v>Accessories</v>
+      </c>
+      <c r="D4" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="E4" s="11" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="F4" s="11" t="str">
+        <v>Available</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="str">
+        <v>INV004</v>
+      </c>
+      <c r="B5" s="11" t="str">
+        <v>Mouse</v>
+      </c>
+      <c r="C5" s="11" t="str">
+        <v>Accessories</v>
+      </c>
+      <c r="D5" s="11" t="n">
+        <v>35</v>
+      </c>
+      <c r="E5" s="11" t="str">
+        <v>Pune</v>
+      </c>
+      <c r="F5" s="11" t="str">
+        <v>Available</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="str">
+        <v>INV005</v>
+      </c>
+      <c r="B6" s="11" t="str">
+        <v>Printer</v>
+      </c>
+      <c r="C6" s="11" t="str">
+        <v>Office Equipment</v>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" s="11" t="str">
+        <v>Chennai</v>
+      </c>
+      <c r="F6" s="11" t="str">
+        <v>Available</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="str">
+        <v>INV006</v>
+      </c>
+      <c r="B7" s="11" t="str">
+        <v>Projector</v>
+      </c>
+      <c r="C7" s="11" t="str">
+        <v>Office Equipment</v>
+      </c>
+      <c r="D7" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="E7" s="11" t="str">
+        <v>Mumbai</v>
+      </c>
+      <c r="F7" s="11" t="str">
+        <v>Available</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="str">
+        <v>INV007</v>
+      </c>
+      <c r="B8" s="11" t="str">
+        <v>Chair</v>
+      </c>
+      <c r="C8" s="11" t="str">
+        <v>Furniture</v>
+      </c>
+      <c r="D8" s="11" t="n">
+        <v>50</v>
+      </c>
+      <c r="E8" s="11" t="str">
+        <v>Delhi</v>
+      </c>
+      <c r="F8" s="11" t="str">
+        <v>Available</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart ns1:id="R65794bffdeb745ea"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>